<commit_message>
Cafetería Móvil: arreglos de la revisión en plan, Word y checklist (M1, M2, M4, m1-m21, m24; M5 parcial con nota y deuda del motor); cifras del caso sin cambios, D9 12/12
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-cafeteria-movil-eventos/checklist-apertura-cafeteria-movil-eventos.xlsx
+++ b/astro-site/public/dl/plan-negocio-cafeteria-movil-eventos/checklist-apertura-cafeteria-movil-eventos.xlsx
@@ -951,8 +951,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, —, N/A. N/A = no aplica, sale del total." type="list">
-      <formula1>"✓,—,N/A"</formula1>
+    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, ☐, N/A. N/A = no aplica, sale del total." type="list">
+      <formula1>"✓,☐,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>El caso del plan es furgoneta + barra-carro: entra en salones y pabellones. El Ape 50 es un ciclomotor (45 km/h como máximo, sin vías rápidas): para ir lejos, en remolque o furgoneta. Compara las tres configuraciones del plan de negocio (sección 6)</t>
+          <t>El caso del plan es furgoneta + barra-carro: entra en salones y pabellones. El Ape 50 es un ciclomotor (45 km/h como máximo, sin vías rápidas): para ir lejos, en remolque o furgoneta. Compara las tres configuraciones del plan de negocio (sección 2)</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Remolque: hasta 750 kg sin matrícula, con tarjeta ITV propia</t>
+          <t>Remolque: hasta 750 kg sin matrícula propia, con tarjeta ITV</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Una nave o un garaje con fregadero para lavar loza, jarras y depósitos, almacén seco y frío, y plaza para la furgoneta. Nada se prepara en casa ni en un trastero sin agua (RD 1021/2022, art. 13.5.b)</t>
+          <t>Una nave o un garaje con fregadero para lavar loza, jarras y depósitos, almacén seco y frío, y plaza para la furgoneta. No se prepara nada en casa para un evento (RD 1021/2022, art. 13.5.b), y un trastero sin agua no sirve para lavar loza ni depósitos</t>
         </is>
       </c>
     </row>
@@ -1490,8 +1490,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18 A19 A20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, —, N/A. N/A = no aplica, sale del total." type="list">
-      <formula1>"✓,—,N/A"</formula1>
+    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18 A19 A20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, ☐, N/A. N/A = no aplica, sale del total." type="list">
+      <formula1>"✓,☐,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
@@ -1975,8 +1975,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, —, N/A. N/A = no aplica, sale del total." type="list">
-      <formula1>"✓,—,N/A"</formula1>
+    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, ☐, N/A. N/A = no aplica, sale del total." type="list">
+      <formula1>"✓,☐,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
@@ -2352,8 +2352,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, —, N/A. N/A = no aplica, sale del total." type="list">
-      <formula1>"✓,—,N/A"</formula1>
+    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, ☐, N/A. N/A = no aplica, sale del total." type="list">
+      <formula1>"✓,☐,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
@@ -2837,8 +2837,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, —, N/A. N/A = no aplica, sale del total." type="list">
-      <formula1>"✓,—,N/A"</formula1>
+    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, ☐, N/A. N/A = no aplica, sale del total." type="list">
+      <formula1>"✓,☐,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Modelo del kit: cancelación en cuatro tramos sin huecos (se retiene el 10, 30, 60 o 100 % menos los costes que te ahorras, y es recíproca), plan B de lluvia (no es fuerza mayor), toma eléctrica y acceso exigidos por escrito al recinto</t>
+          <t>Modelo del kit: cancelación en cuatro tramos sin huecos (se retiene el 10, 30 o 60 %, y en el último el 100 % menos los costes que te ahorras, y es recíproca), plan B de lluvia (no es fuerza mayor), toma eléctrica y acceso exigidos por escrito al recinto</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Ayudante</t>
+          <t>Camarero/a</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Ayudante</t>
+          <t>Camarero/a</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -3322,8 +3322,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, —, N/A. N/A = no aplica, sale del total." type="list">
-      <formula1>"✓,—,N/A"</formula1>
+    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, ☐, N/A. N/A = no aplica, sale del total." type="list">
+      <formula1>"✓,☐,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>

</xml_diff>